<commit_message>
added Docker Set Up
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/OpenCartTestData.xlsx
+++ b/src/test/resources/testdata/OpenCartTestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srava\eclipse-workspace\Sep2025POMSeries\src\test\resouces\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Selenium\Stable\Sep2025POMSeries\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34927BE4-7F02-4E5E-977E-CC74E1F5D4AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB0DA46-163D-416E-B928-84CF5AA84864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{B3C14190-4CE3-4059-84D6-A32B961C35C1}"/>
   </bookViews>

</xml_diff>